<commit_message>
Create Excel File for Login and idp Page Status Check
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/LoginData.xlsx
+++ b/src/test/resources/testdata/LoginData.xlsx
@@ -8,12 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Gyrus_Selenium_Automation\GyrusAim17_Learner_Automation\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{104001FA-8DC2-4220-BB31-8CEC58D9007A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9369F7A4-A0E8-40EF-8E0E-8777DC4A2E31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2688" yWindow="2688" windowWidth="17280" windowHeight="8880" xr2:uid="{C1E078DD-505A-4948-B1DC-386F67C14171}"/>
+    <workbookView xWindow="2688" yWindow="2688" windowWidth="17280" windowHeight="8880" firstSheet="4" activeTab="5" xr2:uid="{C1E078DD-505A-4948-B1DC-386F67C14171}"/>
   </bookViews>
   <sheets>
-    <sheet name="Login" sheetId="1" r:id="rId1"/>
+    <sheet name="ValidLogin" sheetId="1" r:id="rId1"/>
+    <sheet name="FirstTimeLoginRedirectsToChange" sheetId="2" r:id="rId2"/>
+    <sheet name="ValidUserNameAndWrongPass" sheetId="3" r:id="rId3"/>
+    <sheet name="WrongUserNameAndValidPass" sheetId="4" r:id="rId4"/>
+    <sheet name="LastLoginAttemptMessage" sheetId="5" r:id="rId5"/>
+    <sheet name="AccountLockAfterFailedAttempt" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="7">
   <si>
     <t>UserName</t>
   </si>
@@ -45,6 +50,18 @@
   </si>
   <si>
     <t>TTeam01</t>
+  </si>
+  <si>
+    <t>TTeam03</t>
+  </si>
+  <si>
+    <t>tteam07</t>
+  </si>
+  <si>
+    <t>tteam071555</t>
+  </si>
+  <si>
+    <t>tteam08</t>
   </si>
 </sst>
 </file>
@@ -465,4 +482,156 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F7C8116-3211-44A5-AA76-FE583F847690}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2">
+        <v>123</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C280275A-0FF7-40D1-8157-EA566601C65F}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2">
+        <v>123456</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF93B29E-A10A-46E2-AABF-6E2E77E76E0F}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2">
+        <v>123</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3407B8E-64D5-4212-9B31-23BB695B8EDC}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>123545</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A37EEDEC-E2BD-43EB-9D5C-1D96949401F9}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>123</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
minor chanaged in all pages
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/LoginData.xlsx
+++ b/src/test/resources/testdata/LoginData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Gyrus_Selenium_Automation\GyrusAim17_Learner_Automation\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9369F7A4-A0E8-40EF-8E0E-8777DC4A2E31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FDD8973-00D2-4BED-B734-F2919BD87037}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2268" yWindow="2268" windowWidth="17280" windowHeight="8880" xr2:uid="{C1E078DD-505A-4948-B1DC-386F67C14171}"/>
+    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" firstSheet="4" activeTab="4" xr2:uid="{C1E078DD-505A-4948-B1DC-386F67C14171}"/>
   </bookViews>
   <sheets>
     <sheet name="ValidLogin" sheetId="1" r:id="rId1"/>
@@ -49,19 +49,19 @@
     <t>Password</t>
   </si>
   <si>
-    <t>TTeam01</t>
-  </si>
-  <si>
-    <t>TTeam03</t>
-  </si>
-  <si>
-    <t>tteam07</t>
-  </si>
-  <si>
     <t>tteam071555</t>
   </si>
   <si>
-    <t>tteam08</t>
+    <t>p17 student 01</t>
+  </si>
+  <si>
+    <t>p17 student 02</t>
+  </si>
+  <si>
+    <t>p17 student 10</t>
+  </si>
+  <si>
+    <t>p17 student 06</t>
   </si>
 </sst>
 </file>
@@ -459,7 +459,7 @@
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -472,7 +472,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B2">
         <v>123</v>
@@ -489,7 +489,7 @@
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -502,7 +502,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B2">
         <v>123</v>
@@ -519,7 +519,7 @@
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -532,7 +532,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B2">
         <v>123456</v>
@@ -562,7 +562,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B2">
         <v>123</v>
@@ -579,7 +579,7 @@
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -593,10 +593,10 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B2">
-        <v>123545</v>
+        <v>123555</v>
       </c>
     </row>
   </sheetData>
@@ -610,7 +610,7 @@
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -624,10 +624,10 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B2">
-        <v>123</v>
+        <v>123444</v>
       </c>
     </row>
   </sheetData>

</xml_diff>